<commit_message>
Fill HSK1_parts_of_speech_1(1-50).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_1(1-50).xlsx
+++ b/HSK1_parts_of_speech_1(1-50).xlsx
@@ -601,6 +601,16 @@
           <t>любить; любовь</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>любовь</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>любить</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -632,6 +642,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>хобби, увлечение</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>увлекаться, иметь хобби в...</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -658,6 +678,11 @@
           <t>восемь</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>восемь</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -684,6 +709,16 @@
           <t>фразовая частица, выражающая побуждение</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>частица побуждения, предположения («давай», «пожалуй»)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (только в конце предложения)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -710,6 +745,11 @@
           <t>папа</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>папа</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -736,6 +776,16 @@
           <t>белый</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>белый цвет</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>белый; чистый, бесцветный</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -762,6 +812,11 @@
           <t>дневное время</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>дневное время, день</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -788,6 +843,11 @@
           <t>сто</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>сто</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -814,6 +874,11 @@
           <t>группа, класс</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>класс, группа; смена (на работе)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -840,6 +905,16 @@
           <t>половина</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>половина</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>примерно, около (полгода, полтора и т.п.)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -866,6 +941,11 @@
           <t>полгода</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>полгода</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -892,6 +972,11 @@
           <t>полдня</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>полдня; целый день (разг.)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -918,6 +1003,11 @@
           <t>помогать</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>помогать, оказывать помощь кому-л.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -944,6 +1034,16 @@
           <t>помогать; оказывать услугу</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>помогать, оказать услугу (отделяемое: 帮...忙)</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>глагольно-объектная конструкция (离合词)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -970,6 +1070,21 @@
           <t>обертывать; свёрток, сумка</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>свёрток; сумка, мешок</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>оборачивать, заворачивать; упаковывать</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>для свёрнутых/сыпучих в упаковке: пачка, кулёк (一包纸巾)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1001,6 +1116,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>баоцзы, паровой пирожок с начинкой</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1032,6 +1152,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>кубок, чаша (книжн.)</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>для напитков в посуде: стакан, чашка, бокал (一杯水)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1063,6 +1193,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>чашка, стакан</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1089,6 +1224,16 @@
           <t>север; северный</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>север</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>северный</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1115,6 +1260,11 @@
           <t>северная сторона, север</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>северная сторона, север</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1141,6 +1291,11 @@
           <t>Пекин</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Пекин, Бэйцзин</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1172,6 +1327,16 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>корень; основа (книжн.)</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>для предметов с переплётом (книги, тетради, журналы): 一本书</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1203,6 +1368,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>тетрадь</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1229,6 +1399,16 @@
           <t>сравнивать</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>сравнивать (比一比)</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>по сравнению с (他比我高)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1255,6 +1435,21 @@
           <t>не; не надо</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>держать при себе, откладывать (别钱, устар.)</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>другой, прочие (别人, 别的)</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>не надо, не (запрет: 别说话)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1281,6 +1476,16 @@
           <t>другой, иной</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>другие, остальное (其他的)</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>местоимение 别 + частица 的</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1307,6 +1512,16 @@
           <t>другие (люди)</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>человек со стороны</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>другие люди, посторонние</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1333,6 +1548,16 @@
           <t>болезнь</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>болезнь</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>болеть</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1359,6 +1584,11 @@
           <t>больной, пациент</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>больной, пациент</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1385,6 +1615,16 @@
           <t>не (универсальное отрицание)</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>не (универсальное отрицание перед глаголом/прилагательным)</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (только перед сказуемым)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1411,6 +1651,16 @@
           <t>небольшой</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>небольшой</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>отрицательная форма прилагательного (不+大), лексикализованное сочетание</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1437,6 +1687,21 @@
           <t>неверный, неправильный</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>не соответствовать</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>неправильный, неверный</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>отрицательная форма (不+对), устойчивое сочетание</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1463,6 +1728,11 @@
           <t>Не за что!</t>
         </is>
       </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (вежливый ответ «пожалуйста / не за что»); классифицируется как целое</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1489,6 +1759,16 @@
           <t>ни к чему, незачем</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>не нужно, незачем (不用谢)</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>отрицательная глагольная конструкция (不用+V)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1515,6 +1795,11 @@
           <t>овощи; еда, блюдо</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>овощи; блюдо, еда; начинка</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1541,6 +1826,11 @@
           <t>чай</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>чай</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1567,6 +1857,21 @@
           <t>недоставить, не хватать</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>разница, разрыв (差距)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>не доставать, не хватать (还差三块钱); проигрывать (差球)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>плохой, скверный (质量差)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1593,6 +1898,21 @@
           <t>постоянный, частый</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>обыденное, постоянное (книжн.)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>обычный, постоянный (常事)</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>часто (常来)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1619,6 +1939,11 @@
           <t>часто</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>часто, нередко</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1645,6 +1970,11 @@
           <t>петь</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>петь</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1671,6 +2001,16 @@
           <t>петь песню</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>петь песню (отделяемое: 唱...歌)</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>глагольно-объектная конструкция (离合词)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1697,6 +2037,11 @@
           <t>повозка, автомобиль</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>машина, автомобиль; повозка; транспорт</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1723,6 +2068,11 @@
           <t>проездной билет (на колёсном транспорте)</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>проездной билет (на автобус/поезд/метро)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1749,6 +2099,11 @@
           <t>в машине</t>
         </is>
       </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>словосочетание: существительное 车 + постпозиционный локатив 上 («в машине»)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1775,6 +2130,11 @@
           <t>остановка</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>вокзал; остановка, станция</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1801,6 +2161,11 @@
           <t>есть</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>есть, кушать; принимать (пищу)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1827,6 +2192,16 @@
           <t>есть</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>есть, принимать пищу (отделяемое: 吃一顿饭)</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>глагольно-объектная конструкция (离合词)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1853,6 +2228,16 @@
           <t>выходить</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>выходить; выезжать; случаться (出事)</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>для действий/состояний: 出一身汗 (выступить потом)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1879,6 +2264,16 @@
           <t>выходить (сюда)</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>выходить, появляться (движение к говорящему)</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>глагол с направительным дополнением (出来)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1903,6 +2298,16 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>выходить (туда)</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>выходить, уходить (движение от говорящего)</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>глагол с направительным дополнением (出去)</t>
         </is>
       </c>
     </row>

</xml_diff>